<commit_message>
Correction des erreurs remontées lors du review 69cdf84990e7c1914c95963aa4f16bb3f1052474
</commit_message>
<xml_diff>
--- a/SBM-initDocIG/ig/StructureDefinition-fr-core-authenticator.xlsx
+++ b/SBM-initDocIG/ig/StructureDefinition-fr-core-authenticator.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="185">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-01-14T21:51:01+00:00</t>
+    <t>2025-01-15T14:08:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -404,7 +404,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Date/heure de l'attestation de validité </t>
+    <t>Date/heure de l'attestation de validité</t>
   </si>
   <si>
     <t>Authenticator.time.nullFlavor</t>
@@ -417,8 +417,7 @@
 </t>
   </si>
   <si>
-    <t>Date et heure à laquelle le PS atteste la validité des informations portées sur le document. Précisée à la seconde avec précision du décalage 
-par rapport au temps universel (UTC)</t>
+    <t>Date et heure à laquelle le PS atteste la validité des informations portées sur le document. Précisée à la seconde avec précision du décalage par rapport au temps universel (UTC)</t>
   </si>
   <si>
     <t>A quantity specifying a point on the axis of natural time. A point in time is most often represented as a calendar expression.</t>
@@ -430,7 +429,7 @@
     <t>Authenticator.signatureCode</t>
   </si>
   <si>
-    <t>Signature</t>
+    <t>signatureCode signifie que le professionnel a validé les informations portées sur le document.</t>
   </si>
   <si>
     <t>http://hl7.org/cda/stds/core/ValueSet/CDASignatureCode</t>
@@ -444,9 +443,6 @@
   </si>
   <si>
     <t>Authenticator.signatureCode.code</t>
-  </si>
-  <si>
-    <t>S pour 'signed'</t>
   </si>
   <si>
     <t>The plain code symbol defined by the code system. For example, "784.0" is the code symbol of the ICD-9 code "784.0" for headache.</t>
@@ -2696,11 +2692,9 @@
       <c r="K18" t="s" s="2">
         <v>85</v>
       </c>
-      <c r="L18" t="s" s="2">
+      <c r="L18" s="2"/>
+      <c r="M18" t="s" s="2">
         <v>140</v>
-      </c>
-      <c r="M18" t="s" s="2">
-        <v>141</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -2751,7 +2745,7 @@
         <v>74</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>80</v>
@@ -2771,17 +2765,17 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E19" t="s" s="2">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F19" t="s" s="2">
         <v>80</v>
@@ -2803,7 +2797,7 @@
       </c>
       <c r="L19" s="2"/>
       <c r="M19" t="s" s="2">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2854,7 +2848,7 @@
         <v>74</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>80</v>
@@ -2874,17 +2868,17 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E20" t="s" s="2">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F20" t="s" s="2">
         <v>80</v>
@@ -2906,7 +2900,7 @@
       </c>
       <c r="L20" s="2"/>
       <c r="M20" t="s" s="2">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2957,7 +2951,7 @@
         <v>74</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>80</v>
@@ -2977,17 +2971,17 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E21" t="s" s="2">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F21" t="s" s="2">
         <v>80</v>
@@ -3009,7 +3003,7 @@
       </c>
       <c r="L21" s="2"/>
       <c r="M21" t="s" s="2">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3060,7 +3054,7 @@
         <v>74</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>80</v>
@@ -3080,17 +3074,17 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E22" t="s" s="2">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F22" t="s" s="2">
         <v>80</v>
@@ -3112,7 +3106,7 @@
       </c>
       <c r="L22" s="2"/>
       <c r="M22" t="s" s="2">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3163,7 +3157,7 @@
         <v>74</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>80</v>
@@ -3183,10 +3177,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3209,11 +3203,11 @@
         <v>74</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" t="s" s="2">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3264,7 +3258,7 @@
         <v>74</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>80</v>
@@ -3284,10 +3278,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3314,7 +3308,7 @@
       </c>
       <c r="L24" s="2"/>
       <c r="M24" t="s" s="2">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3365,7 +3359,7 @@
         <v>74</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -3385,39 +3379,39 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E25" t="s" s="2">
+        <v>166</v>
+      </c>
+      <c r="F25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G25" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H25" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I25" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="J25" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="K25" t="s" s="2">
         <v>167</v>
-      </c>
-      <c r="F25" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G25" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H25" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I25" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J25" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K25" t="s" s="2">
-        <v>168</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" t="s" s="2">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3468,7 +3462,7 @@
         <v>74</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>
@@ -3488,39 +3482,39 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E26" t="s" s="2">
+        <v>171</v>
+      </c>
+      <c r="F26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G26" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H26" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I26" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="J26" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="K26" t="s" s="2">
         <v>172</v>
-      </c>
-      <c r="F26" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G26" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H26" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I26" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J26" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K26" t="s" s="2">
-        <v>173</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" t="s" s="2">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
@@ -3571,7 +3565,7 @@
         <v>74</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>80</v>
@@ -3591,39 +3585,39 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E27" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="F27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G27" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="H27" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="I27" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="J27" t="s" s="2">
+        <v>74</v>
+      </c>
+      <c r="K27" t="s" s="2">
         <v>177</v>
-      </c>
-      <c r="F27" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G27" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="H27" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I27" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J27" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K27" t="s" s="2">
-        <v>178</v>
       </c>
       <c r="L27" s="2"/>
       <c r="M27" t="s" s="2">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3674,7 +3668,7 @@
         <v>74</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>80</v>
@@ -3694,10 +3688,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3720,11 +3714,11 @@
         <v>74</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L28" s="2"/>
       <c r="M28" t="s" s="2">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -3775,7 +3769,7 @@
         <v>74</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
@@ -3795,10 +3789,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -3821,10 +3815,10 @@
         <v>74</v>
       </c>
       <c r="K29" t="s" s="2">
+        <v>183</v>
+      </c>
+      <c r="L29" t="s" s="2">
         <v>184</v>
-      </c>
-      <c r="L29" t="s" s="2">
-        <v>185</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
@@ -3876,7 +3870,7 @@
         <v>74</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>75</v>

</xml_diff>